<commit_message>
Various evidence screenshots / folder structures
</commit_message>
<xml_diff>
--- a/bench/results/jmeter_S2_analysis.xlsx
+++ b/bench/results/jmeter_S2_analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\corey\Documents\GitHub\Honours-Project\bench\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\corey\Documents\GitHub\Honours-Project\bench\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6064316F-8CB7-4B04-A709-B3DC7FA74FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE1C3C7-0AA5-49E4-B2AE-998686568613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-3480" windowWidth="38640" windowHeight="21120" tabRatio="117" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="117" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3330,16 +3330,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>39.950000000000003</c:v>
+                  <c:v>39.200000000000003</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>41.05</c:v>
+                  <c:v>40.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>41.05</c:v>
+                  <c:v>40.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>41.35</c:v>
+                  <c:v>41</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3417,13 +3417,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>35.5</c:v>
+                  <c:v>35.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>35.5</c:v>
+                  <c:v>35.299999999999997</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>35.5</c:v>
+                  <c:v>35.4</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>35.5</c:v>
@@ -3504,16 +3504,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>38</c:v>
+                  <c:v>37.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>40.85</c:v>
+                  <c:v>39.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>40.85</c:v>
+                  <c:v>40.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>40.85</c:v>
+                  <c:v>40.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3591,16 +3591,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>37.75</c:v>
+                  <c:v>37.200000000000003</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>37.75</c:v>
+                  <c:v>37.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>37.75</c:v>
+                  <c:v>37.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>37.75</c:v>
+                  <c:v>37.700000000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7812,16 +7812,16 @@
         <v>1</v>
       </c>
       <c r="P22" s="6">
-        <v>39.950000000000003</v>
+        <v>39.200000000000003</v>
       </c>
       <c r="Q22" s="6">
-        <v>35.5</v>
+        <v>35.1</v>
       </c>
       <c r="R22" s="6">
-        <v>38</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="S22" s="6">
-        <v>37.75</v>
+        <v>37.200000000000003</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -7844,16 +7844,16 @@
         <v>10</v>
       </c>
       <c r="P23" s="6">
-        <v>41.05</v>
+        <v>40.1</v>
       </c>
       <c r="Q23" s="6">
-        <v>35.5</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="R23" s="6">
-        <v>40.85</v>
+        <v>39.5</v>
       </c>
       <c r="S23" s="6">
-        <v>37.75</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="24" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -7876,16 +7876,16 @@
         <v>50</v>
       </c>
       <c r="P24" s="6">
-        <v>41.05</v>
+        <v>40.5</v>
       </c>
       <c r="Q24" s="6">
-        <v>35.5</v>
+        <v>35.4</v>
       </c>
       <c r="R24" s="6">
-        <v>40.85</v>
+        <v>40.1</v>
       </c>
       <c r="S24" s="6">
-        <v>37.75</v>
+        <v>37.6</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -7908,16 +7908,16 @@
         <v>100</v>
       </c>
       <c r="P25" s="6">
-        <v>41.35</v>
+        <v>41</v>
       </c>
       <c r="Q25" s="6">
         <v>35.5</v>
       </c>
       <c r="R25" s="6">
-        <v>40.85</v>
+        <v>40.4</v>
       </c>
       <c r="S25" s="6">
-        <v>37.75</v>
+        <v>37.700000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>